<commit_message>
added more sorting mechanisms
</commit_message>
<xml_diff>
--- a/Picking by Case ID.xlsx
+++ b/Picking by Case ID.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://dsvcorp-my.sharepoint.com/personal/wendel_santos1_dsv_com/Documents/Documents/code/case-id-barcode-generator/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="51" documentId="8_{33C33F29-AEF1-4D5A-A65C-4D1749FCB150}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E5CC7117-493B-4C84-A8E8-0BB337863359}"/>
+  <xr:revisionPtr revIDLastSave="62" documentId="8_{33C33F29-AEF1-4D5A-A65C-4D1749FCB150}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{22CC86CE-6DA2-4360-BBAB-1533359C8CF5}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="824" uniqueCount="310">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="828" uniqueCount="310">
   <si>
     <t>Order Number</t>
   </si>
@@ -4365,7 +4365,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3EE41E71-179D-477A-9226-D4B51EEC218A}">
   <sheetPr codeName="Sheet2"/>
-  <dimension ref="A1:B108"/>
+  <dimension ref="A1:B112"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
@@ -4714,23 +4714,23 @@
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A44">
-        <v>10226385</v>
+        <v>10226380</v>
       </c>
       <c r="B44" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A45">
-        <v>10226387</v>
+        <v>10226385</v>
       </c>
       <c r="B45" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A46">
-        <v>10226388</v>
+        <v>10226386</v>
       </c>
       <c r="B46" t="s">
         <v>140</v>
@@ -4738,7 +4738,7 @@
     </row>
     <row r="47" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A47">
-        <v>10226392</v>
+        <v>10226387</v>
       </c>
       <c r="B47" t="s">
         <v>140</v>
@@ -4746,7 +4746,7 @@
     </row>
     <row r="48" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A48">
-        <v>10226396</v>
+        <v>10226388</v>
       </c>
       <c r="B48" t="s">
         <v>140</v>
@@ -4754,39 +4754,39 @@
     </row>
     <row r="49" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A49">
-        <v>10226397</v>
+        <v>10226392</v>
       </c>
       <c r="B49" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
     </row>
     <row r="50" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A50">
-        <v>10226398</v>
+        <v>10226396</v>
       </c>
       <c r="B50" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
     </row>
     <row r="51" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A51">
-        <v>10226399</v>
+        <v>10226397</v>
       </c>
       <c r="B51" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
     </row>
     <row r="52" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A52">
-        <v>10226400</v>
+        <v>10226398</v>
       </c>
       <c r="B52" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
     </row>
     <row r="53" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A53">
-        <v>10226401</v>
+        <v>10226399</v>
       </c>
       <c r="B53" t="s">
         <v>140</v>
@@ -4794,39 +4794,39 @@
     </row>
     <row r="54" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A54">
-        <v>10226402</v>
+        <v>10226400</v>
       </c>
       <c r="B54" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
     </row>
     <row r="55" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A55">
-        <v>10226403</v>
+        <v>10226401</v>
       </c>
       <c r="B55" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
     </row>
     <row r="56" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A56">
-        <v>10226405</v>
+        <v>10226402</v>
       </c>
       <c r="B56" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
     </row>
     <row r="57" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A57">
-        <v>10226406</v>
+        <v>10226403</v>
       </c>
       <c r="B57" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
     </row>
     <row r="58" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A58">
-        <v>10226407</v>
+        <v>10226404</v>
       </c>
       <c r="B58" t="s">
         <v>140</v>
@@ -4834,15 +4834,15 @@
     </row>
     <row r="59" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A59">
-        <v>10226409</v>
+        <v>10226405</v>
       </c>
       <c r="B59" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
     </row>
     <row r="60" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A60">
-        <v>10226410</v>
+        <v>10226406</v>
       </c>
       <c r="B60" t="s">
         <v>140</v>
@@ -4850,7 +4850,7 @@
     </row>
     <row r="61" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A61">
-        <v>10226412</v>
+        <v>10226407</v>
       </c>
       <c r="B61" t="s">
         <v>140</v>
@@ -4858,15 +4858,15 @@
     </row>
     <row r="62" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A62">
-        <v>10226413</v>
+        <v>10226409</v>
       </c>
       <c r="B62" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
     </row>
     <row r="63" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A63">
-        <v>10226415</v>
+        <v>10226410</v>
       </c>
       <c r="B63" t="s">
         <v>140</v>
@@ -4874,15 +4874,15 @@
     </row>
     <row r="64" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A64">
-        <v>10226417</v>
+        <v>10226412</v>
       </c>
       <c r="B64" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
     </row>
     <row r="65" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A65">
-        <v>10226418</v>
+        <v>10226413</v>
       </c>
       <c r="B65" t="s">
         <v>140</v>
@@ -4890,23 +4890,23 @@
     </row>
     <row r="66" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A66">
-        <v>10226420</v>
+        <v>10226415</v>
       </c>
       <c r="B66" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
     </row>
     <row r="67" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A67">
-        <v>10226421</v>
+        <v>10226417</v>
       </c>
       <c r="B67" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
     </row>
     <row r="68" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A68">
-        <v>10226422</v>
+        <v>10226418</v>
       </c>
       <c r="B68" t="s">
         <v>140</v>
@@ -4914,39 +4914,39 @@
     </row>
     <row r="69" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A69">
-        <v>10226425</v>
+        <v>10226420</v>
       </c>
       <c r="B69" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
     </row>
     <row r="70" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A70">
-        <v>10226427</v>
+        <v>10226421</v>
       </c>
       <c r="B70" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
     </row>
     <row r="71" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A71">
-        <v>10226429</v>
+        <v>10226422</v>
       </c>
       <c r="B71" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
     </row>
     <row r="72" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A72">
-        <v>10226430</v>
+        <v>10226425</v>
       </c>
       <c r="B72" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
     </row>
     <row r="73" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A73">
-        <v>10226431</v>
+        <v>10226427</v>
       </c>
       <c r="B73" t="s">
         <v>144</v>
@@ -4954,7 +4954,7 @@
     </row>
     <row r="74" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A74">
-        <v>10226432</v>
+        <v>10226429</v>
       </c>
       <c r="B74" t="s">
         <v>144</v>
@@ -4962,31 +4962,31 @@
     </row>
     <row r="75" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A75">
-        <v>10226435</v>
+        <v>10226430</v>
       </c>
       <c r="B75" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
     </row>
     <row r="76" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A76">
-        <v>10226437</v>
+        <v>10226431</v>
       </c>
       <c r="B76" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
     </row>
     <row r="77" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A77">
-        <v>10226438</v>
+        <v>10226432</v>
       </c>
       <c r="B77" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
     </row>
     <row r="78" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A78">
-        <v>10226439</v>
+        <v>10226435</v>
       </c>
       <c r="B78" t="s">
         <v>140</v>
@@ -4994,7 +4994,7 @@
     </row>
     <row r="79" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A79">
-        <v>10226441</v>
+        <v>10226437</v>
       </c>
       <c r="B79" t="s">
         <v>140</v>
@@ -5002,7 +5002,7 @@
     </row>
     <row r="80" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A80">
-        <v>10226442</v>
+        <v>10226438</v>
       </c>
       <c r="B80" t="s">
         <v>140</v>
@@ -5010,7 +5010,7 @@
     </row>
     <row r="81" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A81">
-        <v>10226444</v>
+        <v>10226439</v>
       </c>
       <c r="B81" t="s">
         <v>140</v>
@@ -5018,7 +5018,7 @@
     </row>
     <row r="82" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A82">
-        <v>10226445</v>
+        <v>10226441</v>
       </c>
       <c r="B82" t="s">
         <v>140</v>
@@ -5026,7 +5026,7 @@
     </row>
     <row r="83" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A83">
-        <v>10226446</v>
+        <v>10226442</v>
       </c>
       <c r="B83" t="s">
         <v>140</v>
@@ -5034,7 +5034,7 @@
     </row>
     <row r="84" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A84">
-        <v>10226447</v>
+        <v>10226444</v>
       </c>
       <c r="B84" t="s">
         <v>140</v>
@@ -5042,7 +5042,7 @@
     </row>
     <row r="85" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A85">
-        <v>10226453</v>
+        <v>10226445</v>
       </c>
       <c r="B85" t="s">
         <v>140</v>
@@ -5050,7 +5050,7 @@
     </row>
     <row r="86" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A86">
-        <v>10226454</v>
+        <v>10226446</v>
       </c>
       <c r="B86" t="s">
         <v>140</v>
@@ -5058,7 +5058,7 @@
     </row>
     <row r="87" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A87">
-        <v>10226455</v>
+        <v>10226447</v>
       </c>
       <c r="B87" t="s">
         <v>140</v>
@@ -5066,31 +5066,31 @@
     </row>
     <row r="88" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A88">
-        <v>10226463</v>
+        <v>10226452</v>
       </c>
       <c r="B88" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
     </row>
     <row r="89" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A89">
-        <v>10226618</v>
+        <v>10226453</v>
       </c>
       <c r="B89" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
     </row>
     <row r="90" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A90">
-        <v>10226781</v>
+        <v>10226454</v>
       </c>
       <c r="B90" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
     </row>
     <row r="91" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A91">
-        <v>10227069</v>
+        <v>10226455</v>
       </c>
       <c r="B91" t="s">
         <v>140</v>
@@ -5098,7 +5098,7 @@
     </row>
     <row r="92" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A92">
-        <v>10227309</v>
+        <v>10226463</v>
       </c>
       <c r="B92" t="s">
         <v>144</v>
@@ -5106,7 +5106,7 @@
     </row>
     <row r="93" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A93">
-        <v>10227310</v>
+        <v>10226618</v>
       </c>
       <c r="B93" t="s">
         <v>144</v>
@@ -5114,23 +5114,23 @@
     </row>
     <row r="94" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A94">
-        <v>10227896</v>
+        <v>10226781</v>
       </c>
       <c r="B94" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
     </row>
     <row r="95" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A95">
-        <v>10230675</v>
+        <v>10227069</v>
       </c>
       <c r="B95" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
     </row>
     <row r="96" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A96">
-        <v>10231475</v>
+        <v>10227309</v>
       </c>
       <c r="B96" t="s">
         <v>144</v>
@@ -5138,7 +5138,7 @@
     </row>
     <row r="97" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A97">
-        <v>10231484</v>
+        <v>10227310</v>
       </c>
       <c r="B97" t="s">
         <v>144</v>
@@ -5146,23 +5146,23 @@
     </row>
     <row r="98" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A98">
-        <v>10236617</v>
+        <v>10227896</v>
       </c>
       <c r="B98" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
     </row>
     <row r="99" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A99">
-        <v>10236618</v>
+        <v>10230675</v>
       </c>
       <c r="B99" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
     </row>
     <row r="100" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A100">
-        <v>10236662</v>
+        <v>10231475</v>
       </c>
       <c r="B100" t="s">
         <v>144</v>
@@ -5170,7 +5170,7 @@
     </row>
     <row r="101" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A101">
-        <v>10236672</v>
+        <v>10231484</v>
       </c>
       <c r="B101" t="s">
         <v>144</v>
@@ -5178,15 +5178,15 @@
     </row>
     <row r="102" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A102">
-        <v>10238737</v>
+        <v>10236617</v>
       </c>
       <c r="B102" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
     </row>
     <row r="103" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A103">
-        <v>10242280</v>
+        <v>10236618</v>
       </c>
       <c r="B103" t="s">
         <v>140</v>
@@ -5194,23 +5194,23 @@
     </row>
     <row r="104" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A104">
-        <v>10242291</v>
+        <v>10236662</v>
       </c>
       <c r="B104" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
     </row>
     <row r="105" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A105">
-        <v>10242293</v>
+        <v>10236672</v>
       </c>
       <c r="B105" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
     </row>
     <row r="106" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A106">
-        <v>10247603</v>
+        <v>10238737</v>
       </c>
       <c r="B106" t="s">
         <v>143</v>
@@ -5218,23 +5218,55 @@
     </row>
     <row r="107" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A107">
-        <v>10247604</v>
+        <v>10242280</v>
       </c>
       <c r="B107" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
     </row>
     <row r="108" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A108">
+        <v>10242291</v>
+      </c>
+      <c r="B108" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="109" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A109">
+        <v>10242293</v>
+      </c>
+      <c r="B109" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="110" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A110">
+        <v>10247603</v>
+      </c>
+      <c r="B110" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="111" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A111">
+        <v>10247604</v>
+      </c>
+      <c r="B111" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="112" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A112">
         <v>10247605</v>
       </c>
-      <c r="B108" t="s">
+      <c r="B112" t="s">
         <v>143</v>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:B108" xr:uid="{3EE41E71-179D-477A-9226-D4B51EEC218A}">
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:B108">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:B112">
       <sortCondition ref="A1:A108"/>
     </sortState>
   </autoFilter>
@@ -5324,11 +5356,11 @@
       </c>
       <c r="D4" s="16" t="str">
         <f>IF(Imprimir!B4="", "", _xlfn.XLOOKUP(VALUE(Imprimir!B4),DB!A:A,DB!B:B,""))</f>
-        <v/>
+        <v>BOX</v>
       </c>
       <c r="E4" s="16" t="str">
-        <f>IF(ISBLANK('Colar Pedido'!C2),"",'Colar Pedido'!D2)</f>
-        <v>0000011925</v>
+        <f>IF(ISBLANK('Colar Pedido'!C2),"",'Colar Pedido'!C2)</f>
+        <v>0000118134</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
@@ -5346,11 +5378,11 @@
       </c>
       <c r="D5" s="16" t="str">
         <f>IF(Imprimir!B5="", "", _xlfn.XLOOKUP(VALUE(Imprimir!B5),DB!A:A,DB!B:B,""))</f>
-        <v/>
+        <v>BOX</v>
       </c>
       <c r="E5" s="16" t="str">
-        <f>IF(ISBLANK('Colar Pedido'!C3),"",'Colar Pedido'!D3)</f>
-        <v>0000008709</v>
+        <f>IF(ISBLANK('Colar Pedido'!C3),"",'Colar Pedido'!C3)</f>
+        <v>0000118130</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
@@ -5371,8 +5403,8 @@
         <v>BOX</v>
       </c>
       <c r="E6" s="16" t="str">
-        <f>IF(ISBLANK('Colar Pedido'!C4),"",'Colar Pedido'!D4)</f>
-        <v>0000013709</v>
+        <f>IF(ISBLANK('Colar Pedido'!C4),"",'Colar Pedido'!C4)</f>
+        <v>0000118123</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
@@ -5393,8 +5425,8 @@
         <v>BOX</v>
       </c>
       <c r="E7" s="16" t="str">
-        <f>IF(ISBLANK('Colar Pedido'!C5),"",'Colar Pedido'!D5)</f>
-        <v>0000013830</v>
+        <f>IF(ISBLANK('Colar Pedido'!C5),"",'Colar Pedido'!C5)</f>
+        <v>0000118124</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
@@ -5415,8 +5447,8 @@
         <v>BOX</v>
       </c>
       <c r="E8" s="16" t="str">
-        <f>IF(ISBLANK('Colar Pedido'!C6),"",'Colar Pedido'!D6)</f>
-        <v>0000013563</v>
+        <f>IF(ISBLANK('Colar Pedido'!C6),"",'Colar Pedido'!C6)</f>
+        <v>0000118125</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
@@ -5437,8 +5469,8 @@
         <v>BOX</v>
       </c>
       <c r="E9" s="16" t="str">
-        <f>IF(ISBLANK('Colar Pedido'!C7),"",'Colar Pedido'!D7)</f>
-        <v>0000013019</v>
+        <f>IF(ISBLANK('Colar Pedido'!C7),"",'Colar Pedido'!C7)</f>
+        <v>0000118126</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
@@ -5459,8 +5491,8 @@
         <v>BOX</v>
       </c>
       <c r="E10" s="16" t="str">
-        <f>IF(ISBLANK('Colar Pedido'!C8),"",'Colar Pedido'!D8)</f>
-        <v>0000013833</v>
+        <f>IF(ISBLANK('Colar Pedido'!C8),"",'Colar Pedido'!C8)</f>
+        <v>0000118227</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
@@ -5481,8 +5513,8 @@
         <v>SLIVE</v>
       </c>
       <c r="E11" s="16" t="str">
-        <f>IF(ISBLANK('Colar Pedido'!C9),"",'Colar Pedido'!D9)</f>
-        <v>0000013886</v>
+        <f>IF(ISBLANK('Colar Pedido'!C9),"",'Colar Pedido'!C9)</f>
+        <v>0000118228</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
@@ -5503,8 +5535,8 @@
         <v>SLIVE</v>
       </c>
       <c r="E12" s="16" t="str">
-        <f>IF(ISBLANK('Colar Pedido'!C10),"",'Colar Pedido'!D10)</f>
-        <v>0000013876</v>
+        <f>IF(ISBLANK('Colar Pedido'!C10),"",'Colar Pedido'!C10)</f>
+        <v>0000118229</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
@@ -5525,8 +5557,8 @@
         <v>SLIVE</v>
       </c>
       <c r="E13" s="16" t="str">
-        <f>IF(ISBLANK('Colar Pedido'!C11),"",'Colar Pedido'!D11)</f>
-        <v>0000013835</v>
+        <f>IF(ISBLANK('Colar Pedido'!C11),"",'Colar Pedido'!C11)</f>
+        <v>0000118230</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
@@ -5547,8 +5579,8 @@
         <v>SLIVE</v>
       </c>
       <c r="E14" s="16" t="str">
-        <f>IF(ISBLANK('Colar Pedido'!C12),"",'Colar Pedido'!D12)</f>
-        <v>0000013853</v>
+        <f>IF(ISBLANK('Colar Pedido'!C12),"",'Colar Pedido'!C12)</f>
+        <v>0000118231</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
@@ -5569,8 +5601,8 @@
         <v>SLIVE</v>
       </c>
       <c r="E15" s="16" t="str">
-        <f>IF(ISBLANK('Colar Pedido'!C13),"",'Colar Pedido'!D13)</f>
-        <v>0000013834</v>
+        <f>IF(ISBLANK('Colar Pedido'!C13),"",'Colar Pedido'!C13)</f>
+        <v>0000118232</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
@@ -5591,8 +5623,8 @@
         <v>BOX</v>
       </c>
       <c r="E16" s="16" t="str">
-        <f>IF(ISBLANK('Colar Pedido'!C14),"",'Colar Pedido'!D14)</f>
-        <v>0000013495</v>
+        <f>IF(ISBLANK('Colar Pedido'!C14),"",'Colar Pedido'!C14)</f>
+        <v>0000118233</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
@@ -5613,8 +5645,8 @@
         <v>BOX</v>
       </c>
       <c r="E17" s="16" t="str">
-        <f>IF(ISBLANK('Colar Pedido'!C15),"",'Colar Pedido'!D15)</f>
-        <v>0000010158</v>
+        <f>IF(ISBLANK('Colar Pedido'!C15),"",'Colar Pedido'!C15)</f>
+        <v>0000118234</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
@@ -5635,8 +5667,8 @@
         <v>BOX</v>
       </c>
       <c r="E18" s="16" t="str">
-        <f>IF(ISBLANK('Colar Pedido'!C16),"",'Colar Pedido'!D16)</f>
-        <v>0000013562</v>
+        <f>IF(ISBLANK('Colar Pedido'!C16),"",'Colar Pedido'!C16)</f>
+        <v>0000118235</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
@@ -5657,8 +5689,8 @@
         <v>SLIVE</v>
       </c>
       <c r="E19" s="16" t="str">
-        <f>IF(ISBLANK('Colar Pedido'!C17),"",'Colar Pedido'!D17)</f>
-        <v>0000012489</v>
+        <f>IF(ISBLANK('Colar Pedido'!C17),"",'Colar Pedido'!C17)</f>
+        <v>0000118236</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
@@ -5679,8 +5711,8 @@
         <v>BOX</v>
       </c>
       <c r="E20" s="16" t="str">
-        <f>IF(ISBLANK('Colar Pedido'!C18),"",'Colar Pedido'!D18)</f>
-        <v>0000013896</v>
+        <f>IF(ISBLANK('Colar Pedido'!C18),"",'Colar Pedido'!C18)</f>
+        <v>0000118237</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
@@ -5701,8 +5733,8 @@
         <v>SLIVE</v>
       </c>
       <c r="E21" s="16" t="str">
-        <f>IF(ISBLANK('Colar Pedido'!C19),"",'Colar Pedido'!D19)</f>
-        <v>0000014043</v>
+        <f>IF(ISBLANK('Colar Pedido'!C19),"",'Colar Pedido'!C19)</f>
+        <v>0000118238</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
@@ -5723,8 +5755,8 @@
         <v>SLIVE</v>
       </c>
       <c r="E22" s="16" t="str">
-        <f>IF(ISBLANK('Colar Pedido'!C20),"",'Colar Pedido'!D20)</f>
-        <v>0000014043</v>
+        <f>IF(ISBLANK('Colar Pedido'!C20),"",'Colar Pedido'!C20)</f>
+        <v>0000118239</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
@@ -5745,8 +5777,8 @@
         <v>SLIVE</v>
       </c>
       <c r="E23" s="16" t="str">
-        <f>IF(ISBLANK('Colar Pedido'!C21),"",'Colar Pedido'!D21)</f>
-        <v>0000014066</v>
+        <f>IF(ISBLANK('Colar Pedido'!C21),"",'Colar Pedido'!C21)</f>
+        <v>0000118240</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
@@ -5767,8 +5799,8 @@
         <v>BOX</v>
       </c>
       <c r="E24" s="16" t="str">
-        <f>IF(ISBLANK('Colar Pedido'!C22),"",'Colar Pedido'!D22)</f>
-        <v>0000011465</v>
+        <f>IF(ISBLANK('Colar Pedido'!C22),"",'Colar Pedido'!C22)</f>
+        <v>0000118241</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
@@ -5789,8 +5821,8 @@
         <v>BOX</v>
       </c>
       <c r="E25" s="16" t="str">
-        <f>IF(ISBLANK('Colar Pedido'!C23),"",'Colar Pedido'!D23)</f>
-        <v>0000013467</v>
+        <f>IF(ISBLANK('Colar Pedido'!C23),"",'Colar Pedido'!C23)</f>
+        <v>0000118242</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
@@ -5811,8 +5843,8 @@
         <v>BOX</v>
       </c>
       <c r="E26" s="16" t="str">
-        <f>IF(ISBLANK('Colar Pedido'!C24),"",'Colar Pedido'!D24)</f>
-        <v>0000009496</v>
+        <f>IF(ISBLANK('Colar Pedido'!C24),"",'Colar Pedido'!C24)</f>
+        <v>0000118243</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
@@ -5833,8 +5865,8 @@
         <v/>
       </c>
       <c r="E27" s="16" t="str">
-        <f>IF(ISBLANK('Colar Pedido'!C25),"",'Colar Pedido'!D25)</f>
-        <v>0000013869</v>
+        <f>IF(ISBLANK('Colar Pedido'!C25),"",'Colar Pedido'!C25)</f>
+        <v>0000118244</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
@@ -5855,8 +5887,8 @@
         <v>SLIVE</v>
       </c>
       <c r="E28" s="16" t="str">
-        <f>IF(ISBLANK('Colar Pedido'!C26),"",'Colar Pedido'!D26)</f>
-        <v>0000014064</v>
+        <f>IF(ISBLANK('Colar Pedido'!C26),"",'Colar Pedido'!C26)</f>
+        <v>0000118245</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
@@ -5874,11 +5906,11 @@
       </c>
       <c r="D29" s="16" t="str">
         <f>IF(Imprimir!B29="", "", _xlfn.XLOOKUP(VALUE(Imprimir!B29),DB!A:A,DB!B:B,""))</f>
-        <v/>
+        <v>SLEEVE P</v>
       </c>
       <c r="E29" s="16" t="str">
-        <f>IF(ISBLANK('Colar Pedido'!C27),"",'Colar Pedido'!D27)</f>
-        <v>0000013843</v>
+        <f>IF(ISBLANK('Colar Pedido'!C27),"",'Colar Pedido'!C27)</f>
+        <v>0000118246</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
@@ -5896,11 +5928,11 @@
       </c>
       <c r="D30" s="16" t="str">
         <f>IF(Imprimir!B30="", "", _xlfn.XLOOKUP(VALUE(Imprimir!B30),DB!A:A,DB!B:B,""))</f>
-        <v/>
+        <v>SLEEVE P</v>
       </c>
       <c r="E30" s="16" t="str">
-        <f>IF(ISBLANK('Colar Pedido'!C28),"",'Colar Pedido'!D28)</f>
-        <v>0000013859</v>
+        <f>IF(ISBLANK('Colar Pedido'!C28),"",'Colar Pedido'!C28)</f>
+        <v>0000118247</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
@@ -5918,11 +5950,11 @@
       </c>
       <c r="D31" s="16" t="str">
         <f>IF(Imprimir!B31="", "", _xlfn.XLOOKUP(VALUE(Imprimir!B31),DB!A:A,DB!B:B,""))</f>
-        <v/>
+        <v>SLEEVE P</v>
       </c>
       <c r="E31" s="16" t="str">
-        <f>IF(ISBLANK('Colar Pedido'!C29),"",'Colar Pedido'!D29)</f>
-        <v>0000013841</v>
+        <f>IF(ISBLANK('Colar Pedido'!C29),"",'Colar Pedido'!C29)</f>
+        <v>0000118248</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
@@ -5943,8 +5975,8 @@
         <v>SLIVE</v>
       </c>
       <c r="E32" s="16" t="str">
-        <f>IF(ISBLANK('Colar Pedido'!C30),"",'Colar Pedido'!D30)</f>
-        <v>0000013851</v>
+        <f>IF(ISBLANK('Colar Pedido'!C30),"",'Colar Pedido'!C30)</f>
+        <v>0000118249</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
@@ -5962,11 +5994,11 @@
       </c>
       <c r="D33" s="16" t="str">
         <f>IF(Imprimir!B33="", "", _xlfn.XLOOKUP(VALUE(Imprimir!B33),DB!A:A,DB!B:B,""))</f>
-        <v/>
+        <v>BOX</v>
       </c>
       <c r="E33" s="16" t="str">
-        <f>IF(ISBLANK('Colar Pedido'!C31),"",'Colar Pedido'!D31)</f>
-        <v>0000013863</v>
+        <f>IF(ISBLANK('Colar Pedido'!C31),"",'Colar Pedido'!C31)</f>
+        <v>0000118250</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.25">
@@ -5984,11 +6016,11 @@
       </c>
       <c r="D34" s="16" t="str">
         <f>IF(Imprimir!B34="", "", _xlfn.XLOOKUP(VALUE(Imprimir!B34),DB!A:A,DB!B:B,""))</f>
-        <v/>
+        <v>BOX</v>
       </c>
       <c r="E34" s="16" t="str">
-        <f>IF(ISBLANK('Colar Pedido'!C32),"",'Colar Pedido'!D32)</f>
-        <v>0000013870</v>
+        <f>IF(ISBLANK('Colar Pedido'!C32),"",'Colar Pedido'!C32)</f>
+        <v>0000118251</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
@@ -6006,11 +6038,11 @@
       </c>
       <c r="D35" s="16" t="str">
         <f>IF(Imprimir!B35="", "", _xlfn.XLOOKUP(VALUE(Imprimir!B35),DB!A:A,DB!B:B,""))</f>
-        <v/>
+        <v>BOX</v>
       </c>
       <c r="E35" s="16" t="str">
-        <f>IF(ISBLANK('Colar Pedido'!C33),"",'Colar Pedido'!D33)</f>
-        <v>0000013883</v>
+        <f>IF(ISBLANK('Colar Pedido'!C33),"",'Colar Pedido'!C33)</f>
+        <v>0000118252</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.25">
@@ -6028,11 +6060,11 @@
       </c>
       <c r="D36" s="16" t="str">
         <f>IF(Imprimir!B36="", "", _xlfn.XLOOKUP(VALUE(Imprimir!B36),DB!A:A,DB!B:B,""))</f>
-        <v/>
+        <v>BOX</v>
       </c>
       <c r="E36" s="16" t="str">
-        <f>IF(ISBLANK('Colar Pedido'!C34),"",'Colar Pedido'!D34)</f>
-        <v>0000013706</v>
+        <f>IF(ISBLANK('Colar Pedido'!C34),"",'Colar Pedido'!C34)</f>
+        <v>0000118253</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.25">
@@ -6053,8 +6085,8 @@
         <v>BOX</v>
       </c>
       <c r="E37" s="16" t="str">
-        <f>IF(ISBLANK('Colar Pedido'!C35),"",'Colar Pedido'!D35)</f>
-        <v>0000013837</v>
+        <f>IF(ISBLANK('Colar Pedido'!C35),"",'Colar Pedido'!C35)</f>
+        <v>0000118254</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.25">
@@ -6075,8 +6107,8 @@
         <v>BOX</v>
       </c>
       <c r="E38" s="16" t="str">
-        <f>IF(ISBLANK('Colar Pedido'!C36),"",'Colar Pedido'!D36)</f>
-        <v>0000011775</v>
+        <f>IF(ISBLANK('Colar Pedido'!C36),"",'Colar Pedido'!C36)</f>
+        <v>0000118255</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.25">
@@ -6097,8 +6129,8 @@
         <v>BOX</v>
       </c>
       <c r="E39" s="16" t="str">
-        <f>IF(ISBLANK('Colar Pedido'!C37),"",'Colar Pedido'!D37)</f>
-        <v>0000013840</v>
+        <f>IF(ISBLANK('Colar Pedido'!C37),"",'Colar Pedido'!C37)</f>
+        <v>0000118256</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.25">
@@ -6119,8 +6151,8 @@
         <v>SLIVE</v>
       </c>
       <c r="E40" s="16" t="str">
-        <f>IF(ISBLANK('Colar Pedido'!C38),"",'Colar Pedido'!D38)</f>
-        <v>0000013728</v>
+        <f>IF(ISBLANK('Colar Pedido'!C38),"",'Colar Pedido'!C38)</f>
+        <v>0000118257</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.25">
@@ -6141,8 +6173,8 @@
         <v>SLEEVE P</v>
       </c>
       <c r="E41" s="16" t="str">
-        <f>IF(ISBLANK('Colar Pedido'!C39),"",'Colar Pedido'!D39)</f>
-        <v>0000013735</v>
+        <f>IF(ISBLANK('Colar Pedido'!C39),"",'Colar Pedido'!C39)</f>
+        <v>0000118258</v>
       </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.25">
@@ -6163,8 +6195,8 @@
         <v>NINE</v>
       </c>
       <c r="E42" s="16" t="str">
-        <f>IF(ISBLANK('Colar Pedido'!C40),"",'Colar Pedido'!D40)</f>
-        <v>0000013438</v>
+        <f>IF(ISBLANK('Colar Pedido'!C40),"",'Colar Pedido'!C40)</f>
+        <v>0000118259</v>
       </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.25">
@@ -6185,8 +6217,8 @@
         <v>NINE</v>
       </c>
       <c r="E43" s="16" t="str">
-        <f>IF(ISBLANK('Colar Pedido'!C41),"",'Colar Pedido'!D41)</f>
-        <v>0000013942</v>
+        <f>IF(ISBLANK('Colar Pedido'!C41),"",'Colar Pedido'!C41)</f>
+        <v>0000118260</v>
       </c>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.25">
@@ -6207,8 +6239,8 @@
         <v>BOX</v>
       </c>
       <c r="E44" s="16" t="str">
-        <f>IF(ISBLANK('Colar Pedido'!C42),"",'Colar Pedido'!D42)</f>
-        <v>0000013436</v>
+        <f>IF(ISBLANK('Colar Pedido'!C42),"",'Colar Pedido'!C42)</f>
+        <v>0000118261</v>
       </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.25">
@@ -6229,8 +6261,8 @@
         <v>BOX</v>
       </c>
       <c r="E45" s="16" t="str">
-        <f>IF(ISBLANK('Colar Pedido'!C43),"",'Colar Pedido'!D43)</f>
-        <v>0000012543</v>
+        <f>IF(ISBLANK('Colar Pedido'!C43),"",'Colar Pedido'!C43)</f>
+        <v>0000118262</v>
       </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.25">
@@ -6251,8 +6283,8 @@
         <v>BOX</v>
       </c>
       <c r="E46" s="16" t="str">
-        <f>IF(ISBLANK('Colar Pedido'!C44),"",'Colar Pedido'!D44)</f>
-        <v>0000012647</v>
+        <f>IF(ISBLANK('Colar Pedido'!C44),"",'Colar Pedido'!C44)</f>
+        <v>0000118263</v>
       </c>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.25">
@@ -6270,11 +6302,11 @@
       </c>
       <c r="D47" s="16" t="str">
         <f>IF(Imprimir!B47="", "", _xlfn.XLOOKUP(VALUE(Imprimir!B47),DB!A:A,DB!B:B,""))</f>
-        <v/>
+        <v>BOX</v>
       </c>
       <c r="E47" s="16" t="str">
-        <f>IF(ISBLANK('Colar Pedido'!C45),"",'Colar Pedido'!D45)</f>
-        <v>0000013912</v>
+        <f>IF(ISBLANK('Colar Pedido'!C45),"",'Colar Pedido'!C45)</f>
+        <v>0000118264</v>
       </c>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.25">
@@ -6295,8 +6327,8 @@
         <v/>
       </c>
       <c r="E48" s="16" t="str">
-        <f>IF(ISBLANK('Colar Pedido'!C46),"",'Colar Pedido'!D46)</f>
-        <v>0000013088</v>
+        <f>IF(ISBLANK('Colar Pedido'!C46),"",'Colar Pedido'!C46)</f>
+        <v>0000118265</v>
       </c>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.25">
@@ -6317,8 +6349,8 @@
         <v/>
       </c>
       <c r="E49" s="16" t="str">
-        <f>IF(ISBLANK('Colar Pedido'!C47),"",'Colar Pedido'!D47)</f>
-        <v>0000013088</v>
+        <f>IF(ISBLANK('Colar Pedido'!C47),"",'Colar Pedido'!C47)</f>
+        <v>0000118266</v>
       </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.25">
@@ -6336,11 +6368,11 @@
       </c>
       <c r="D50" s="16" t="str">
         <f>IF(Imprimir!B50="", "", _xlfn.XLOOKUP(VALUE(Imprimir!B50),DB!A:A,DB!B:B,""))</f>
-        <v/>
+        <v>BOX</v>
       </c>
       <c r="E50" s="16" t="str">
-        <f>IF(ISBLANK('Colar Pedido'!C48),"",'Colar Pedido'!D48)</f>
-        <v>0000013864</v>
+        <f>IF(ISBLANK('Colar Pedido'!C48),"",'Colar Pedido'!C48)</f>
+        <v>0000118267</v>
       </c>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.25">
@@ -6361,7 +6393,7 @@
         <v/>
       </c>
       <c r="E51" s="16" t="str">
-        <f>IF(ISBLANK('Colar Pedido'!C49),"",'Colar Pedido'!D49)</f>
+        <f>IF(ISBLANK('Colar Pedido'!C49),"",'Colar Pedido'!C49)</f>
         <v/>
       </c>
     </row>
@@ -6383,7 +6415,7 @@
         <v/>
       </c>
       <c r="E52" s="16" t="str">
-        <f>IF(ISBLANK('Colar Pedido'!C50),"",'Colar Pedido'!D50)</f>
+        <f>IF(ISBLANK('Colar Pedido'!C50),"",'Colar Pedido'!C50)</f>
         <v/>
       </c>
     </row>
@@ -6405,7 +6437,7 @@
         <v/>
       </c>
       <c r="E53" s="16" t="str">
-        <f>IF(ISBLANK('Colar Pedido'!C51),"",'Colar Pedido'!D51)</f>
+        <f>IF(ISBLANK('Colar Pedido'!C51),"",'Colar Pedido'!C51)</f>
         <v/>
       </c>
     </row>
@@ -6427,7 +6459,7 @@
         <v/>
       </c>
       <c r="E54" s="16" t="str">
-        <f>IF(ISBLANK('Colar Pedido'!C52),"",'Colar Pedido'!D52)</f>
+        <f>IF(ISBLANK('Colar Pedido'!C52),"",'Colar Pedido'!C52)</f>
         <v/>
       </c>
     </row>
@@ -6449,7 +6481,7 @@
         <v/>
       </c>
       <c r="E55" s="16" t="str">
-        <f>IF(ISBLANK('Colar Pedido'!C53),"",'Colar Pedido'!D53)</f>
+        <f>IF(ISBLANK('Colar Pedido'!C53),"",'Colar Pedido'!C53)</f>
         <v/>
       </c>
     </row>
@@ -6471,7 +6503,7 @@
         <v/>
       </c>
       <c r="E56" s="16" t="str">
-        <f>IF(ISBLANK('Colar Pedido'!C54),"",'Colar Pedido'!D54)</f>
+        <f>IF(ISBLANK('Colar Pedido'!C54),"",'Colar Pedido'!C54)</f>
         <v/>
       </c>
     </row>
@@ -6493,7 +6525,7 @@
         <v/>
       </c>
       <c r="E57" s="16" t="str">
-        <f>IF(ISBLANK('Colar Pedido'!C55),"",'Colar Pedido'!D55)</f>
+        <f>IF(ISBLANK('Colar Pedido'!C55),"",'Colar Pedido'!C55)</f>
         <v/>
       </c>
     </row>
@@ -6515,7 +6547,7 @@
         <v/>
       </c>
       <c r="E58" s="16" t="str">
-        <f>IF(ISBLANK('Colar Pedido'!C56),"",'Colar Pedido'!D56)</f>
+        <f>IF(ISBLANK('Colar Pedido'!C56),"",'Colar Pedido'!C56)</f>
         <v/>
       </c>
     </row>
@@ -6537,7 +6569,7 @@
         <v/>
       </c>
       <c r="E59" s="16" t="str">
-        <f>IF(ISBLANK('Colar Pedido'!C57),"",'Colar Pedido'!D57)</f>
+        <f>IF(ISBLANK('Colar Pedido'!C57),"",'Colar Pedido'!C57)</f>
         <v/>
       </c>
     </row>
@@ -6559,7 +6591,7 @@
         <v/>
       </c>
       <c r="E60" s="16" t="str">
-        <f>IF(ISBLANK('Colar Pedido'!C58),"",'Colar Pedido'!D58)</f>
+        <f>IF(ISBLANK('Colar Pedido'!C58),"",'Colar Pedido'!C58)</f>
         <v/>
       </c>
     </row>
@@ -6581,7 +6613,7 @@
         <v/>
       </c>
       <c r="E61" s="16" t="str">
-        <f>IF(ISBLANK('Colar Pedido'!C59),"",'Colar Pedido'!D59)</f>
+        <f>IF(ISBLANK('Colar Pedido'!C59),"",'Colar Pedido'!C59)</f>
         <v/>
       </c>
     </row>
@@ -6603,7 +6635,7 @@
         <v/>
       </c>
       <c r="E62" s="16" t="str">
-        <f>IF(ISBLANK('Colar Pedido'!C60),"",'Colar Pedido'!D60)</f>
+        <f>IF(ISBLANK('Colar Pedido'!C60),"",'Colar Pedido'!C60)</f>
         <v/>
       </c>
     </row>
@@ -6625,7 +6657,7 @@
         <v/>
       </c>
       <c r="E63" s="16" t="str">
-        <f>IF(ISBLANK('Colar Pedido'!C61),"",'Colar Pedido'!D61)</f>
+        <f>IF(ISBLANK('Colar Pedido'!C61),"",'Colar Pedido'!C61)</f>
         <v/>
       </c>
     </row>
@@ -6647,7 +6679,7 @@
         <v/>
       </c>
       <c r="E64" s="16" t="str">
-        <f>IF(ISBLANK('Colar Pedido'!C62),"",'Colar Pedido'!D62)</f>
+        <f>IF(ISBLANK('Colar Pedido'!C62),"",'Colar Pedido'!C62)</f>
         <v/>
       </c>
     </row>
@@ -6669,7 +6701,7 @@
         <v/>
       </c>
       <c r="E65" s="16" t="str">
-        <f>IF(ISBLANK('Colar Pedido'!C63),"",'Colar Pedido'!D63)</f>
+        <f>IF(ISBLANK('Colar Pedido'!C63),"",'Colar Pedido'!C63)</f>
         <v/>
       </c>
     </row>
@@ -6691,7 +6723,7 @@
         <v/>
       </c>
       <c r="E66" s="16" t="str">
-        <f>IF(ISBLANK('Colar Pedido'!C64),"",'Colar Pedido'!D64)</f>
+        <f>IF(ISBLANK('Colar Pedido'!C64),"",'Colar Pedido'!C64)</f>
         <v/>
       </c>
     </row>
@@ -6713,7 +6745,7 @@
         <v/>
       </c>
       <c r="E67" s="16" t="str">
-        <f>IF(ISBLANK('Colar Pedido'!C65),"",'Colar Pedido'!D65)</f>
+        <f>IF(ISBLANK('Colar Pedido'!C65),"",'Colar Pedido'!C65)</f>
         <v/>
       </c>
     </row>
@@ -6735,7 +6767,7 @@
         <v/>
       </c>
       <c r="E68" s="16" t="str">
-        <f>IF(ISBLANK('Colar Pedido'!C66),"",'Colar Pedido'!D66)</f>
+        <f>IF(ISBLANK('Colar Pedido'!C66),"",'Colar Pedido'!C66)</f>
         <v/>
       </c>
     </row>
@@ -6757,7 +6789,7 @@
         <v/>
       </c>
       <c r="E69" s="16" t="str">
-        <f>IF(ISBLANK('Colar Pedido'!C67),"",'Colar Pedido'!D67)</f>
+        <f>IF(ISBLANK('Colar Pedido'!C67),"",'Colar Pedido'!C67)</f>
         <v/>
       </c>
     </row>
@@ -6779,7 +6811,7 @@
         <v/>
       </c>
       <c r="E70" s="16" t="str">
-        <f>IF(ISBLANK('Colar Pedido'!C68),"",'Colar Pedido'!D68)</f>
+        <f>IF(ISBLANK('Colar Pedido'!C68),"",'Colar Pedido'!C68)</f>
         <v/>
       </c>
     </row>
@@ -6801,7 +6833,7 @@
         <v/>
       </c>
       <c r="E71" s="16" t="str">
-        <f>IF(ISBLANK('Colar Pedido'!C69),"",'Colar Pedido'!D69)</f>
+        <f>IF(ISBLANK('Colar Pedido'!C69),"",'Colar Pedido'!C69)</f>
         <v/>
       </c>
     </row>
@@ -6823,7 +6855,7 @@
         <v/>
       </c>
       <c r="E72" s="16" t="str">
-        <f>IF(ISBLANK('Colar Pedido'!C70),"",'Colar Pedido'!D70)</f>
+        <f>IF(ISBLANK('Colar Pedido'!C70),"",'Colar Pedido'!C70)</f>
         <v/>
       </c>
     </row>
@@ -6845,7 +6877,7 @@
         <v/>
       </c>
       <c r="E73" s="16" t="str">
-        <f>IF(ISBLANK('Colar Pedido'!C71),"",'Colar Pedido'!D71)</f>
+        <f>IF(ISBLANK('Colar Pedido'!C71),"",'Colar Pedido'!C71)</f>
         <v/>
       </c>
     </row>
@@ -6867,7 +6899,7 @@
         <v/>
       </c>
       <c r="E74" s="16" t="str">
-        <f>IF(ISBLANK('Colar Pedido'!C72),"",'Colar Pedido'!D72)</f>
+        <f>IF(ISBLANK('Colar Pedido'!C72),"",'Colar Pedido'!C72)</f>
         <v/>
       </c>
     </row>
@@ -6889,7 +6921,7 @@
         <v/>
       </c>
       <c r="E75" s="16" t="str">
-        <f>IF(ISBLANK('Colar Pedido'!C73),"",'Colar Pedido'!D73)</f>
+        <f>IF(ISBLANK('Colar Pedido'!C73),"",'Colar Pedido'!C73)</f>
         <v/>
       </c>
     </row>
@@ -6911,7 +6943,7 @@
         <v/>
       </c>
       <c r="E76" s="16" t="str">
-        <f>IF(ISBLANK('Colar Pedido'!C74),"",'Colar Pedido'!D74)</f>
+        <f>IF(ISBLANK('Colar Pedido'!C74),"",'Colar Pedido'!C74)</f>
         <v/>
       </c>
     </row>
@@ -6933,7 +6965,7 @@
         <v/>
       </c>
       <c r="E77" s="16" t="str">
-        <f>IF(ISBLANK('Colar Pedido'!C75),"",'Colar Pedido'!D75)</f>
+        <f>IF(ISBLANK('Colar Pedido'!C75),"",'Colar Pedido'!C75)</f>
         <v/>
       </c>
     </row>
@@ -6955,7 +6987,7 @@
         <v/>
       </c>
       <c r="E78" s="16" t="str">
-        <f>IF(ISBLANK('Colar Pedido'!C76),"",'Colar Pedido'!D76)</f>
+        <f>IF(ISBLANK('Colar Pedido'!C76),"",'Colar Pedido'!C76)</f>
         <v/>
       </c>
     </row>
@@ -6977,7 +7009,7 @@
         <v/>
       </c>
       <c r="E79" s="16" t="str">
-        <f>IF(ISBLANK('Colar Pedido'!C77),"",'Colar Pedido'!D77)</f>
+        <f>IF(ISBLANK('Colar Pedido'!C77),"",'Colar Pedido'!C77)</f>
         <v/>
       </c>
     </row>
@@ -6999,7 +7031,7 @@
         <v/>
       </c>
       <c r="E80" s="16" t="str">
-        <f>IF(ISBLANK('Colar Pedido'!C78),"",'Colar Pedido'!D78)</f>
+        <f>IF(ISBLANK('Colar Pedido'!C78),"",'Colar Pedido'!C78)</f>
         <v/>
       </c>
     </row>
@@ -7021,7 +7053,7 @@
         <v/>
       </c>
       <c r="E81" s="16" t="str">
-        <f>IF(ISBLANK('Colar Pedido'!C79),"",'Colar Pedido'!D79)</f>
+        <f>IF(ISBLANK('Colar Pedido'!C79),"",'Colar Pedido'!C79)</f>
         <v/>
       </c>
     </row>
@@ -7043,7 +7075,7 @@
         <v/>
       </c>
       <c r="E82" s="16" t="str">
-        <f>IF(ISBLANK('Colar Pedido'!C80),"",'Colar Pedido'!D80)</f>
+        <f>IF(ISBLANK('Colar Pedido'!C80),"",'Colar Pedido'!C80)</f>
         <v/>
       </c>
     </row>
@@ -7065,7 +7097,7 @@
         <v/>
       </c>
       <c r="E83" s="16" t="str">
-        <f>IF(ISBLANK('Colar Pedido'!C81),"",'Colar Pedido'!D81)</f>
+        <f>IF(ISBLANK('Colar Pedido'!C81),"",'Colar Pedido'!C81)</f>
         <v/>
       </c>
     </row>
@@ -7087,7 +7119,7 @@
         <v/>
       </c>
       <c r="E84" s="16" t="str">
-        <f>IF(ISBLANK('Colar Pedido'!C82),"",'Colar Pedido'!D82)</f>
+        <f>IF(ISBLANK('Colar Pedido'!C82),"",'Colar Pedido'!C82)</f>
         <v/>
       </c>
     </row>
@@ -7109,7 +7141,7 @@
         <v/>
       </c>
       <c r="E85" s="16" t="str">
-        <f>IF(ISBLANK('Colar Pedido'!C83),"",'Colar Pedido'!D83)</f>
+        <f>IF(ISBLANK('Colar Pedido'!C83),"",'Colar Pedido'!C83)</f>
         <v/>
       </c>
     </row>
@@ -7131,7 +7163,7 @@
         <v/>
       </c>
       <c r="E86" s="16" t="str">
-        <f>IF(ISBLANK('Colar Pedido'!C84),"",'Colar Pedido'!D84)</f>
+        <f>IF(ISBLANK('Colar Pedido'!C84),"",'Colar Pedido'!C84)</f>
         <v/>
       </c>
     </row>
@@ -7153,7 +7185,7 @@
         <v/>
       </c>
       <c r="E87" s="16" t="str">
-        <f>IF(ISBLANK('Colar Pedido'!C85),"",'Colar Pedido'!D85)</f>
+        <f>IF(ISBLANK('Colar Pedido'!C85),"",'Colar Pedido'!C85)</f>
         <v/>
       </c>
     </row>
@@ -7175,7 +7207,7 @@
         <v/>
       </c>
       <c r="E88" s="16" t="str">
-        <f>IF(ISBLANK('Colar Pedido'!C86),"",'Colar Pedido'!D86)</f>
+        <f>IF(ISBLANK('Colar Pedido'!C86),"",'Colar Pedido'!C86)</f>
         <v/>
       </c>
     </row>
@@ -7197,7 +7229,7 @@
         <v/>
       </c>
       <c r="E89" s="16" t="str">
-        <f>IF(ISBLANK('Colar Pedido'!C87),"",'Colar Pedido'!D87)</f>
+        <f>IF(ISBLANK('Colar Pedido'!C87),"",'Colar Pedido'!C87)</f>
         <v/>
       </c>
     </row>
@@ -7219,7 +7251,7 @@
         <v/>
       </c>
       <c r="E90" s="16" t="str">
-        <f>IF(ISBLANK('Colar Pedido'!C88),"",'Colar Pedido'!D88)</f>
+        <f>IF(ISBLANK('Colar Pedido'!C88),"",'Colar Pedido'!C88)</f>
         <v/>
       </c>
     </row>
@@ -7241,7 +7273,7 @@
         <v/>
       </c>
       <c r="E91" s="16" t="str">
-        <f>IF(ISBLANK('Colar Pedido'!C89),"",'Colar Pedido'!D89)</f>
+        <f>IF(ISBLANK('Colar Pedido'!C89),"",'Colar Pedido'!C89)</f>
         <v/>
       </c>
     </row>
@@ -7263,7 +7295,7 @@
         <v/>
       </c>
       <c r="E92" s="16" t="str">
-        <f>IF(ISBLANK('Colar Pedido'!C90),"",'Colar Pedido'!D90)</f>
+        <f>IF(ISBLANK('Colar Pedido'!C90),"",'Colar Pedido'!C90)</f>
         <v/>
       </c>
     </row>
@@ -7285,7 +7317,7 @@
         <v/>
       </c>
       <c r="E93" s="16" t="str">
-        <f>IF(ISBLANK('Colar Pedido'!C91),"",'Colar Pedido'!D91)</f>
+        <f>IF(ISBLANK('Colar Pedido'!C91),"",'Colar Pedido'!C91)</f>
         <v/>
       </c>
     </row>
@@ -7307,7 +7339,7 @@
         <v/>
       </c>
       <c r="E94" s="16" t="str">
-        <f>IF(ISBLANK('Colar Pedido'!C92),"",'Colar Pedido'!D92)</f>
+        <f>IF(ISBLANK('Colar Pedido'!C92),"",'Colar Pedido'!C92)</f>
         <v/>
       </c>
     </row>
@@ -7329,7 +7361,7 @@
         <v/>
       </c>
       <c r="E95" s="16" t="str">
-        <f>IF(ISBLANK('Colar Pedido'!C93),"",'Colar Pedido'!D93)</f>
+        <f>IF(ISBLANK('Colar Pedido'!C93),"",'Colar Pedido'!C93)</f>
         <v/>
       </c>
     </row>
@@ -7351,7 +7383,7 @@
         <v/>
       </c>
       <c r="E96" s="16" t="str">
-        <f>IF(ISBLANK('Colar Pedido'!C94),"",'Colar Pedido'!D94)</f>
+        <f>IF(ISBLANK('Colar Pedido'!C94),"",'Colar Pedido'!C94)</f>
         <v/>
       </c>
     </row>
@@ -7373,7 +7405,7 @@
         <v/>
       </c>
       <c r="E97" s="16" t="str">
-        <f>IF(ISBLANK('Colar Pedido'!C95),"",'Colar Pedido'!D95)</f>
+        <f>IF(ISBLANK('Colar Pedido'!C95),"",'Colar Pedido'!C95)</f>
         <v/>
       </c>
     </row>
@@ -7395,7 +7427,7 @@
         <v/>
       </c>
       <c r="E98" s="16" t="str">
-        <f>IF(ISBLANK('Colar Pedido'!C96),"",'Colar Pedido'!D96)</f>
+        <f>IF(ISBLANK('Colar Pedido'!C96),"",'Colar Pedido'!C96)</f>
         <v/>
       </c>
     </row>
@@ -7417,7 +7449,7 @@
         <v/>
       </c>
       <c r="E99" s="16" t="str">
-        <f>IF(ISBLANK('Colar Pedido'!C97),"",'Colar Pedido'!D97)</f>
+        <f>IF(ISBLANK('Colar Pedido'!C97),"",'Colar Pedido'!C97)</f>
         <v/>
       </c>
     </row>
@@ -7439,7 +7471,7 @@
         <v/>
       </c>
       <c r="E100" s="16" t="str">
-        <f>IF(ISBLANK('Colar Pedido'!C98),"",'Colar Pedido'!D98)</f>
+        <f>IF(ISBLANK('Colar Pedido'!C98),"",'Colar Pedido'!C98)</f>
         <v/>
       </c>
     </row>
@@ -7461,7 +7493,7 @@
         <v/>
       </c>
       <c r="E101" s="16" t="str">
-        <f>IF(ISBLANK('Colar Pedido'!C99),"",'Colar Pedido'!D99)</f>
+        <f>IF(ISBLANK('Colar Pedido'!C99),"",'Colar Pedido'!C99)</f>
         <v/>
       </c>
     </row>

</xml_diff>